<commit_message>
new similarity results, with addition
</commit_message>
<xml_diff>
--- a/all_sim/det_gemini_domain.xlsx
+++ b/all_sim/det_gemini_domain.xlsx
@@ -331,16 +331,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="36.300000000000004" min="1" max="1" bestFit="1" customWidth="1"/>
-    <col width="24.200000000000003" min="2" max="2" bestFit="1" customWidth="1"/>
-    <col width="24.200000000000003" min="3" max="3" bestFit="1" customWidth="1"/>
-    <col width="24.200000000000003" min="4" max="4" bestFit="1" customWidth="1"/>
-    <col width="24.200000000000003" min="5" max="5" bestFit="1" customWidth="1"/>
+    <col width="23.1" min="2" max="2" bestFit="1" customWidth="1"/>
+    <col width="23.1" min="3" max="3" bestFit="1" customWidth="1"/>
+    <col width="23.1" min="4" max="4" bestFit="1" customWidth="1"/>
+    <col width="23.1" min="5" max="5" bestFit="1" customWidth="1"/>
     <col width="24.200000000000003" min="6" max="6" bestFit="1" customWidth="1"/>
-    <col width="24.200000000000003" min="7" max="7" bestFit="1" customWidth="1"/>
-    <col width="25.3" min="8" max="8" bestFit="1" customWidth="1"/>
-    <col width="25.3" min="9" max="9" bestFit="1" customWidth="1"/>
-    <col width="25.3" min="10" max="10" bestFit="1" customWidth="1"/>
-    <col width="25.3" min="11" max="11" bestFit="1" customWidth="1"/>
+    <col width="23.1" min="7" max="7" bestFit="1" customWidth="1"/>
+    <col width="23.1" min="8" max="8" bestFit="1" customWidth="1"/>
+    <col width="23.1" min="9" max="9" bestFit="1" customWidth="1"/>
+    <col width="24.200000000000003" min="10" max="10" bestFit="1" customWidth="1"/>
+    <col width="23.1" min="11" max="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -350,34 +350,34 @@
         </is>
       </c>
       <c r="B1" s="0" t="n">
-        <v>0.2421875</v>
+        <v>0.62109375</v>
       </c>
       <c r="C1" s="0" t="n">
-        <v>0.2421875</v>
+        <v>0.62109375</v>
       </c>
       <c r="D1" s="0" t="n">
-        <v>0.2421875</v>
+        <v>0.62109375</v>
       </c>
       <c r="E1" s="0" t="n">
-        <v>0.2421875</v>
+        <v>0.62109375</v>
       </c>
       <c r="F1" s="0" t="n">
-        <v>0.2421875</v>
+        <v>0.62109375</v>
       </c>
       <c r="G1" s="0" t="n">
-        <v>0.2421875</v>
+        <v>0.62109375</v>
       </c>
       <c r="H1" s="0" t="n">
-        <v>0.2421875</v>
+        <v>0.62109375</v>
       </c>
       <c r="I1" s="0" t="n">
-        <v>0.2421875</v>
+        <v>0.62109375</v>
       </c>
       <c r="J1" s="0" t="n">
-        <v>0.2421875</v>
+        <v>0.62109375</v>
       </c>
       <c r="K1" s="0" t="n">
-        <v>0.2421875</v>
+        <v>0.62109375</v>
       </c>
     </row>
     <row r="2">
@@ -387,34 +387,34 @@
         </is>
       </c>
       <c r="B2" s="0" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.4437830687830688</v>
       </c>
       <c r="C2" s="0" t="n">
-        <v>0.2</v>
+        <v>0.5537037037037037</v>
       </c>
       <c r="D2" s="0" t="n">
-        <v>0.2</v>
+        <v>0.5537037037037037</v>
       </c>
       <c r="E2" s="0" t="n">
-        <v>0.2</v>
+        <v>0.5537037037037037</v>
       </c>
       <c r="F2" s="0" t="n">
-        <v>0.2</v>
+        <v>0.5537037037037037</v>
       </c>
       <c r="G2" s="0" t="n">
-        <v>0.2</v>
+        <v>0.5537037037037037</v>
       </c>
       <c r="H2" s="0" t="n">
-        <v>0.028095238095238097</v>
+        <v>0.439047619047619</v>
       </c>
       <c r="I2" s="0" t="n">
-        <v>0.028095238095238097</v>
+        <v>0.4694047619047619</v>
       </c>
       <c r="J2" s="0" t="n">
-        <v>0.028095238095238097</v>
+        <v>0.4694047619047619</v>
       </c>
       <c r="K2" s="0" t="n">
-        <v>0.014341085271317831</v>
+        <v>0.3563084736701417</v>
       </c>
     </row>
     <row r="3">
@@ -424,34 +424,34 @@
         </is>
       </c>
       <c r="B3" s="0" t="n">
-        <v>0.42857142857142855</v>
+        <v>0.680952380952381</v>
       </c>
       <c r="C3" s="0" t="n">
-        <v>0.42857142857142855</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="D3" s="0" t="n">
-        <v>0.42857142857142855</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="E3" s="0" t="n">
-        <v>0.42857142857142855</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="F3" s="0" t="n">
-        <v>0.42857142857142855</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="G3" s="0" t="n">
-        <v>0.42857142857142855</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="H3" s="0" t="n">
-        <v>0.42857142857142855</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="I3" s="0" t="n">
-        <v>0.42857142857142855</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="J3" s="0" t="n">
-        <v>0.42857142857142855</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="K3" s="0" t="n">
-        <v>0.42857142857142855</v>
+        <v>0.7142857142857143</v>
       </c>
     </row>
     <row r="4">
@@ -461,34 +461,34 @@
         </is>
       </c>
       <c r="B4" s="0" t="n">
-        <v>0.3240740740740741</v>
+        <v>0.6179193899782135</v>
       </c>
       <c r="C4" s="0" t="n">
-        <v>0.3240740740740741</v>
+        <v>0.6179193899782135</v>
       </c>
       <c r="D4" s="0" t="n">
-        <v>0.44444444444444453</v>
+        <v>0.7065972222222223</v>
       </c>
       <c r="E4" s="0" t="n">
-        <v>0.44444444444444453</v>
+        <v>0.7065972222222223</v>
       </c>
       <c r="F4" s="0" t="n">
-        <v>0.44444444444444453</v>
+        <v>0.7065972222222223</v>
       </c>
       <c r="G4" s="0" t="n">
-        <v>0.44444444444444453</v>
+        <v>0.7065972222222223</v>
       </c>
       <c r="H4" s="0" t="n">
-        <v>0.44444444444444453</v>
+        <v>0.7065972222222223</v>
       </c>
       <c r="I4" s="0" t="n">
-        <v>0.44444444444444453</v>
+        <v>0.7065972222222223</v>
       </c>
       <c r="J4" s="0" t="n">
-        <v>0.44444444444444453</v>
+        <v>0.7065972222222223</v>
       </c>
       <c r="K4" s="0" t="n">
-        <v>0.44444444444444453</v>
+        <v>0.7065972222222223</v>
       </c>
     </row>
     <row r="5">
@@ -498,34 +498,34 @@
         </is>
       </c>
       <c r="B5" s="0" t="n">
-        <v>0.8452380952380952</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="C5" s="0" t="n">
-        <v>0.8452380952380952</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="D5" s="0" t="n">
-        <v>0.8452380952380952</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="E5" s="0" t="n">
-        <v>0.8452380952380952</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="F5" s="0" t="n">
-        <v>0.8452380952380952</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="G5" s="0" t="n">
-        <v>0.8452380952380952</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="H5" s="0" t="n">
-        <v>0.8452380952380952</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="I5" s="0" t="n">
-        <v>0.8452380952380952</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="J5" s="0" t="n">
-        <v>0.8452380952380952</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="K5" s="0" t="n">
-        <v>0.8452380952380952</v>
+        <v>0.9226190476190477</v>
       </c>
     </row>
     <row r="6">
@@ -535,34 +535,34 @@
         </is>
       </c>
       <c r="B6" s="0" t="n">
-        <v>1.0</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="C6" s="0" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.9166666666666667</v>
       </c>
       <c r="D6" s="0" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.9166666666666667</v>
       </c>
       <c r="E6" s="0" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.9166666666666667</v>
       </c>
       <c r="F6" s="0" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.9166666666666667</v>
       </c>
       <c r="G6" s="0" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.9166666666666667</v>
       </c>
       <c r="H6" s="0" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.9166666666666667</v>
       </c>
       <c r="I6" s="0" t="n">
-        <v>0.7416666666666667</v>
+        <v>0.8708333333333333</v>
       </c>
       <c r="J6" s="0" t="n">
-        <v>0.7416666666666667</v>
+        <v>0.8708333333333333</v>
       </c>
       <c r="K6" s="0" t="n">
-        <v>0.7083333333333334</v>
+        <v>0.8541666666666667</v>
       </c>
     </row>
     <row r="7">
@@ -575,31 +575,31 @@
         <v>1.0</v>
       </c>
       <c r="C7" s="0" t="n">
-        <v>0.9249999999999999</v>
+        <v>0.9624999999999999</v>
       </c>
       <c r="D7" s="0" t="n">
-        <v>0.9249999999999999</v>
+        <v>0.9624999999999999</v>
       </c>
       <c r="E7" s="0" t="n">
-        <v>0.9249999999999999</v>
+        <v>0.9624999999999999</v>
       </c>
       <c r="F7" s="0" t="n">
-        <v>0.9249999999999999</v>
+        <v>0.9624999999999999</v>
       </c>
       <c r="G7" s="0" t="n">
-        <v>0.9249999999999999</v>
+        <v>0.9624999999999999</v>
       </c>
       <c r="H7" s="0" t="n">
-        <v>0.9249999999999999</v>
+        <v>0.9624999999999999</v>
       </c>
       <c r="I7" s="0" t="n">
-        <v>0.9249999999999999</v>
+        <v>0.9624999999999999</v>
       </c>
       <c r="J7" s="0" t="n">
-        <v>0.6357142857142857</v>
+        <v>0.8178571428571428</v>
       </c>
       <c r="K7" s="0" t="n">
-        <v>0.6662698412698412</v>
+        <v>0.8331349206349206</v>
       </c>
     </row>
     <row r="8">
@@ -609,34 +609,34 @@
         </is>
       </c>
       <c r="B8" s="0" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
       <c r="C8" s="0" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
       <c r="D8" s="0" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
       <c r="E8" s="0" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
       <c r="F8" s="0" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
       <c r="G8" s="0" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
       <c r="H8" s="0" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
       <c r="I8" s="0" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
       <c r="J8" s="0" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
       <c r="K8" s="0" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="9">
@@ -652,28 +652,28 @@
         <v>1.0</v>
       </c>
       <c r="D9" s="0" t="n">
-        <v>1.0</v>
+        <v>0.9473684210526316</v>
       </c>
       <c r="E9" s="0" t="n">
-        <v>1.0</v>
+        <v>0.9473684210526316</v>
       </c>
       <c r="F9" s="0" t="n">
-        <v>1.0</v>
+        <v>0.9473684210526316</v>
       </c>
       <c r="G9" s="0" t="n">
-        <v>1.0</v>
+        <v>0.9473684210526316</v>
       </c>
       <c r="H9" s="0" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9153846153846155</v>
       </c>
       <c r="I9" s="0" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9153846153846155</v>
       </c>
       <c r="J9" s="0" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9153846153846155</v>
       </c>
       <c r="K9" s="0" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9153846153846155</v>
       </c>
     </row>
     <row r="10">
@@ -683,34 +683,34 @@
         </is>
       </c>
       <c r="B10" s="0" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.8436293436293436</v>
       </c>
       <c r="C10" s="0" t="n">
-        <v>0.9523809523809524</v>
+        <v>0.9293154761904763</v>
       </c>
       <c r="D10" s="0" t="n">
-        <v>0.8783068783068783</v>
+        <v>0.8922784391534391</v>
       </c>
       <c r="E10" s="0" t="n">
-        <v>0.8783068783068783</v>
+        <v>0.8922784391534391</v>
       </c>
       <c r="F10" s="0" t="n">
-        <v>0.8783068783068783</v>
+        <v>0.8922784391534391</v>
       </c>
       <c r="G10" s="0" t="n">
-        <v>0.8783068783068783</v>
+        <v>0.8922784391534391</v>
       </c>
       <c r="H10" s="0" t="n">
-        <v>0.8783068783068783</v>
+        <v>0.8922784391534391</v>
       </c>
       <c r="I10" s="0" t="n">
-        <v>0.8783068783068783</v>
+        <v>0.8922784391534391</v>
       </c>
       <c r="J10" s="0" t="n">
-        <v>0.8783068783068783</v>
+        <v>0.8922784391534391</v>
       </c>
       <c r="K10" s="0" t="n">
-        <v>0.8783068783068783</v>
+        <v>0.8922784391534391</v>
       </c>
     </row>
     <row r="11">
@@ -720,34 +720,34 @@
         </is>
       </c>
       <c r="B11" s="0" t="n">
-        <v>0.746031746031746</v>
+        <v>0.8502886002886003</v>
       </c>
       <c r="C11" s="0" t="n">
-        <v>0.580952380952381</v>
+        <v>0.7256613756613757</v>
       </c>
       <c r="D11" s="0" t="n">
-        <v>0.3959899749373434</v>
+        <v>0.5194235588972431</v>
       </c>
       <c r="E11" s="0" t="n">
-        <v>0.0981684981684982</v>
+        <v>0.343003168003168</v>
       </c>
       <c r="F11" s="0" t="n">
-        <v>0.10351089588377727</v>
+        <v>0.34737588589809304</v>
       </c>
       <c r="G11" s="0" t="n">
-        <v>0.20402298850574713</v>
+        <v>0.402896450005086</v>
       </c>
       <c r="H11" s="0" t="n">
-        <v>0.303921568627451</v>
+        <v>0.5066119471044231</v>
       </c>
       <c r="I11" s="0" t="n">
-        <v>0.303921568627451</v>
+        <v>0.5370959194488607</v>
       </c>
       <c r="J11" s="0" t="n">
-        <v>0.22883597883597886</v>
+        <v>0.49955312455312456</v>
       </c>
       <c r="K11" s="0" t="n">
-        <v>0.34803921568627455</v>
+        <v>0.5724571078431373</v>
       </c>
     </row>
     <row r="12">
@@ -757,34 +757,34 @@
         </is>
       </c>
       <c r="B12" s="0" t="n">
-        <v>0.8</v>
+        <v>0.8534883720930233</v>
       </c>
       <c r="C12" s="0" t="n">
-        <v>0.8</v>
+        <v>0.7823529411764706</v>
       </c>
       <c r="D12" s="0" t="n">
-        <v>0.8</v>
+        <v>0.8534883720930233</v>
       </c>
       <c r="E12" s="0" t="n">
-        <v>0.8</v>
+        <v>0.8534883720930233</v>
       </c>
       <c r="F12" s="0" t="n">
-        <v>0.8</v>
+        <v>0.8534883720930233</v>
       </c>
       <c r="G12" s="0" t="n">
-        <v>0.8</v>
+        <v>0.8534883720930233</v>
       </c>
       <c r="H12" s="0" t="n">
-        <v>0.8</v>
+        <v>0.8534883720930233</v>
       </c>
       <c r="I12" s="0" t="n">
-        <v>0.8</v>
+        <v>0.8534883720930233</v>
       </c>
       <c r="J12" s="0" t="n">
-        <v>0.8</v>
+        <v>0.8534883720930233</v>
       </c>
       <c r="K12" s="0" t="n">
-        <v>0.8</v>
+        <v>0.8534883720930233</v>
       </c>
     </row>
     <row r="13">
@@ -794,34 +794,34 @@
         </is>
       </c>
       <c r="B13" s="0" t="n">
-        <v>0.71875</v>
+        <v>0.828125</v>
       </c>
       <c r="C13" s="0" t="n">
-        <v>0.66875</v>
+        <v>0.8040719696969697</v>
       </c>
       <c r="D13" s="0" t="n">
-        <v>0.66875</v>
+        <v>0.8040719696969697</v>
       </c>
       <c r="E13" s="0" t="n">
-        <v>0.66875</v>
+        <v>0.8040719696969697</v>
       </c>
       <c r="F13" s="0" t="n">
-        <v>0.66875</v>
+        <v>0.8040719696969697</v>
       </c>
       <c r="G13" s="0" t="n">
-        <v>0.66875</v>
+        <v>0.8040719696969697</v>
       </c>
       <c r="H13" s="0" t="n">
-        <v>0.66875</v>
+        <v>0.8040719696969697</v>
       </c>
       <c r="I13" s="0" t="n">
-        <v>0.66875</v>
+        <v>0.8040719696969697</v>
       </c>
       <c r="J13" s="0" t="n">
-        <v>0.66875</v>
+        <v>0.8040719696969697</v>
       </c>
       <c r="K13" s="0" t="n">
-        <v>0.66875</v>
+        <v>0.8040719696969697</v>
       </c>
     </row>
     <row r="14">
@@ -831,34 +831,34 @@
         </is>
       </c>
       <c r="B14" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.9613095238095238</v>
       </c>
       <c r="C14" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.9613095238095238</v>
       </c>
       <c r="D14" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.9613095238095238</v>
       </c>
       <c r="E14" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.9613095238095238</v>
       </c>
       <c r="F14" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.9613095238095238</v>
       </c>
       <c r="G14" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.9613095238095238</v>
       </c>
       <c r="H14" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.9613095238095238</v>
       </c>
       <c r="I14" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.9613095238095238</v>
       </c>
       <c r="J14" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.9613095238095238</v>
       </c>
       <c r="K14" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.9613095238095238</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
add Multiplicative aggragation into final ts for the control flow penalty
</commit_message>
<xml_diff>
--- a/all_sim/det_gemini_domain.xlsx
+++ b/all_sim/det_gemini_domain.xlsx
@@ -331,16 +331,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="36.300000000000004" min="1" max="1" bestFit="1" customWidth="1"/>
-    <col width="23.1" min="2" max="2" bestFit="1" customWidth="1"/>
-    <col width="23.1" min="3" max="3" bestFit="1" customWidth="1"/>
-    <col width="23.1" min="4" max="4" bestFit="1" customWidth="1"/>
-    <col width="23.1" min="5" max="5" bestFit="1" customWidth="1"/>
+    <col width="24.200000000000003" min="2" max="2" bestFit="1" customWidth="1"/>
+    <col width="24.200000000000003" min="3" max="3" bestFit="1" customWidth="1"/>
+    <col width="24.200000000000003" min="4" max="4" bestFit="1" customWidth="1"/>
+    <col width="24.200000000000003" min="5" max="5" bestFit="1" customWidth="1"/>
     <col width="24.200000000000003" min="6" max="6" bestFit="1" customWidth="1"/>
-    <col width="23.1" min="7" max="7" bestFit="1" customWidth="1"/>
-    <col width="23.1" min="8" max="8" bestFit="1" customWidth="1"/>
-    <col width="23.1" min="9" max="9" bestFit="1" customWidth="1"/>
-    <col width="24.200000000000003" min="10" max="10" bestFit="1" customWidth="1"/>
-    <col width="23.1" min="11" max="11" bestFit="1" customWidth="1"/>
+    <col width="24.200000000000003" min="7" max="7" bestFit="1" customWidth="1"/>
+    <col width="24.200000000000003" min="8" max="8" bestFit="1" customWidth="1"/>
+    <col width="25.3" min="9" max="9" bestFit="1" customWidth="1"/>
+    <col width="25.3" min="10" max="10" bestFit="1" customWidth="1"/>
+    <col width="25.3" min="11" max="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -350,34 +350,34 @@
         </is>
       </c>
       <c r="B1" s="0" t="n">
-        <v>0.62109375</v>
+        <v>0.2421875</v>
       </c>
       <c r="C1" s="0" t="n">
-        <v>0.62109375</v>
+        <v>0.2421875</v>
       </c>
       <c r="D1" s="0" t="n">
-        <v>0.62109375</v>
+        <v>0.2421875</v>
       </c>
       <c r="E1" s="0" t="n">
-        <v>0.62109375</v>
+        <v>0.2421875</v>
       </c>
       <c r="F1" s="0" t="n">
-        <v>0.62109375</v>
+        <v>0.2421875</v>
       </c>
       <c r="G1" s="0" t="n">
-        <v>0.62109375</v>
+        <v>0.2421875</v>
       </c>
       <c r="H1" s="0" t="n">
-        <v>0.62109375</v>
+        <v>0.2421875</v>
       </c>
       <c r="I1" s="0" t="n">
-        <v>0.62109375</v>
+        <v>0.2421875</v>
       </c>
       <c r="J1" s="0" t="n">
-        <v>0.62109375</v>
+        <v>0.2421875</v>
       </c>
       <c r="K1" s="0" t="n">
-        <v>0.62109375</v>
+        <v>0.2421875</v>
       </c>
     </row>
     <row r="2">
@@ -387,34 +387,34 @@
         </is>
       </c>
       <c r="B2" s="0" t="n">
-        <v>0.4437830687830688</v>
+        <v>0.03042328042328042</v>
       </c>
       <c r="C2" s="0" t="n">
-        <v>0.5537037037037037</v>
+        <v>0.1814814814814815</v>
       </c>
       <c r="D2" s="0" t="n">
-        <v>0.5537037037037037</v>
+        <v>0.1814814814814815</v>
       </c>
       <c r="E2" s="0" t="n">
-        <v>0.5537037037037037</v>
+        <v>0.1814814814814815</v>
       </c>
       <c r="F2" s="0" t="n">
-        <v>0.5537037037037037</v>
+        <v>0.1814814814814815</v>
       </c>
       <c r="G2" s="0" t="n">
-        <v>0.5537037037037037</v>
+        <v>0.1814814814814815</v>
       </c>
       <c r="H2" s="0" t="n">
-        <v>0.439047619047619</v>
+        <v>0.02388095238095238</v>
       </c>
       <c r="I2" s="0" t="n">
-        <v>0.4694047619047619</v>
+        <v>0.025586734693877553</v>
       </c>
       <c r="J2" s="0" t="n">
-        <v>0.4694047619047619</v>
+        <v>0.025586734693877553</v>
       </c>
       <c r="K2" s="0" t="n">
-        <v>0.3563084736701417</v>
+        <v>0.010014033680834002</v>
       </c>
     </row>
     <row r="3">
@@ -424,34 +424,34 @@
         </is>
       </c>
       <c r="B3" s="0" t="n">
-        <v>0.680952380952381</v>
+        <v>0.39999999999999997</v>
       </c>
       <c r="C3" s="0" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.42857142857142855</v>
       </c>
       <c r="D3" s="0" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.42857142857142855</v>
       </c>
       <c r="E3" s="0" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.42857142857142855</v>
       </c>
       <c r="F3" s="0" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.42857142857142855</v>
       </c>
       <c r="G3" s="0" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.42857142857142855</v>
       </c>
       <c r="H3" s="0" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.42857142857142855</v>
       </c>
       <c r="I3" s="0" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.42857142857142855</v>
       </c>
       <c r="J3" s="0" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.42857142857142855</v>
       </c>
       <c r="K3" s="0" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.42857142857142855</v>
       </c>
     </row>
     <row r="4">
@@ -461,34 +461,34 @@
         </is>
       </c>
       <c r="B4" s="0" t="n">
-        <v>0.6179193899782135</v>
+        <v>0.29547930283224405</v>
       </c>
       <c r="C4" s="0" t="n">
-        <v>0.6179193899782135</v>
+        <v>0.29547930283224405</v>
       </c>
       <c r="D4" s="0" t="n">
-        <v>0.7065972222222223</v>
+        <v>0.43055555555555564</v>
       </c>
       <c r="E4" s="0" t="n">
-        <v>0.7065972222222223</v>
+        <v>0.43055555555555564</v>
       </c>
       <c r="F4" s="0" t="n">
-        <v>0.7065972222222223</v>
+        <v>0.43055555555555564</v>
       </c>
       <c r="G4" s="0" t="n">
-        <v>0.7065972222222223</v>
+        <v>0.43055555555555564</v>
       </c>
       <c r="H4" s="0" t="n">
-        <v>0.7065972222222223</v>
+        <v>0.43055555555555564</v>
       </c>
       <c r="I4" s="0" t="n">
-        <v>0.7065972222222223</v>
+        <v>0.43055555555555564</v>
       </c>
       <c r="J4" s="0" t="n">
-        <v>0.7065972222222223</v>
+        <v>0.43055555555555564</v>
       </c>
       <c r="K4" s="0" t="n">
-        <v>0.7065972222222223</v>
+        <v>0.43055555555555564</v>
       </c>
     </row>
     <row r="5">
@@ -498,34 +498,34 @@
         </is>
       </c>
       <c r="B5" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.8452380952380952</v>
       </c>
       <c r="C5" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.8452380952380952</v>
       </c>
       <c r="D5" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.8452380952380952</v>
       </c>
       <c r="E5" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.8452380952380952</v>
       </c>
       <c r="F5" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.8452380952380952</v>
       </c>
       <c r="G5" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.8452380952380952</v>
       </c>
       <c r="H5" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.8452380952380952</v>
       </c>
       <c r="I5" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.8452380952380952</v>
       </c>
       <c r="J5" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.8452380952380952</v>
       </c>
       <c r="K5" s="0" t="n">
-        <v>0.9226190476190477</v>
+        <v>0.8452380952380952</v>
       </c>
     </row>
     <row r="6">
@@ -535,34 +535,34 @@
         </is>
       </c>
       <c r="B6" s="0" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="C6" s="0" t="n">
-        <v>0.9166666666666667</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="D6" s="0" t="n">
-        <v>0.9166666666666667</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E6" s="0" t="n">
-        <v>0.9166666666666667</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F6" s="0" t="n">
-        <v>0.9166666666666667</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="G6" s="0" t="n">
-        <v>0.9166666666666667</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="H6" s="0" t="n">
-        <v>0.9166666666666667</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="I6" s="0" t="n">
-        <v>0.8708333333333333</v>
+        <v>0.7416666666666667</v>
       </c>
       <c r="J6" s="0" t="n">
-        <v>0.8708333333333333</v>
+        <v>0.7416666666666667</v>
       </c>
       <c r="K6" s="0" t="n">
-        <v>0.8541666666666667</v>
+        <v>0.7083333333333334</v>
       </c>
     </row>
     <row r="7">
@@ -575,31 +575,31 @@
         <v>1.0</v>
       </c>
       <c r="C7" s="0" t="n">
-        <v>0.9624999999999999</v>
+        <v>0.9249999999999999</v>
       </c>
       <c r="D7" s="0" t="n">
-        <v>0.9624999999999999</v>
+        <v>0.9249999999999999</v>
       </c>
       <c r="E7" s="0" t="n">
-        <v>0.9624999999999999</v>
+        <v>0.9249999999999999</v>
       </c>
       <c r="F7" s="0" t="n">
-        <v>0.9624999999999999</v>
+        <v>0.9249999999999999</v>
       </c>
       <c r="G7" s="0" t="n">
-        <v>0.9624999999999999</v>
+        <v>0.9249999999999999</v>
       </c>
       <c r="H7" s="0" t="n">
-        <v>0.9624999999999999</v>
+        <v>0.9249999999999999</v>
       </c>
       <c r="I7" s="0" t="n">
-        <v>0.9624999999999999</v>
+        <v>0.9249999999999999</v>
       </c>
       <c r="J7" s="0" t="n">
-        <v>0.8178571428571428</v>
+        <v>0.6357142857142857</v>
       </c>
       <c r="K7" s="0" t="n">
-        <v>0.8331349206349206</v>
+        <v>0.6662698412698412</v>
       </c>
     </row>
     <row r="8">
@@ -609,34 +609,34 @@
         </is>
       </c>
       <c r="B8" s="0" t="n">
-        <v>0.8</v>
+        <v>0.6222222222222222</v>
       </c>
       <c r="C8" s="0" t="n">
-        <v>0.8</v>
+        <v>0.6222222222222222</v>
       </c>
       <c r="D8" s="0" t="n">
-        <v>0.8</v>
+        <v>0.6222222222222222</v>
       </c>
       <c r="E8" s="0" t="n">
-        <v>0.8</v>
+        <v>0.6222222222222222</v>
       </c>
       <c r="F8" s="0" t="n">
-        <v>0.8</v>
+        <v>0.6222222222222222</v>
       </c>
       <c r="G8" s="0" t="n">
-        <v>0.8</v>
+        <v>0.6222222222222222</v>
       </c>
       <c r="H8" s="0" t="n">
-        <v>0.8</v>
+        <v>0.6222222222222222</v>
       </c>
       <c r="I8" s="0" t="n">
-        <v>0.8</v>
+        <v>0.6222222222222222</v>
       </c>
       <c r="J8" s="0" t="n">
-        <v>0.8</v>
+        <v>0.6222222222222222</v>
       </c>
       <c r="K8" s="0" t="n">
-        <v>0.8</v>
+        <v>0.6222222222222222</v>
       </c>
     </row>
     <row r="9">
@@ -652,28 +652,28 @@
         <v>1.0</v>
       </c>
       <c r="D9" s="0" t="n">
-        <v>0.9473684210526316</v>
+        <v>0.8947368421052632</v>
       </c>
       <c r="E9" s="0" t="n">
-        <v>0.9473684210526316</v>
+        <v>0.8947368421052632</v>
       </c>
       <c r="F9" s="0" t="n">
-        <v>0.9473684210526316</v>
+        <v>0.8947368421052632</v>
       </c>
       <c r="G9" s="0" t="n">
-        <v>0.9473684210526316</v>
+        <v>0.8947368421052632</v>
       </c>
       <c r="H9" s="0" t="n">
-        <v>0.9153846153846155</v>
+        <v>0.8376068376068376</v>
       </c>
       <c r="I9" s="0" t="n">
-        <v>0.9153846153846155</v>
+        <v>0.8376068376068376</v>
       </c>
       <c r="J9" s="0" t="n">
-        <v>0.9153846153846155</v>
+        <v>0.8376068376068376</v>
       </c>
       <c r="K9" s="0" t="n">
-        <v>0.9153846153846155</v>
+        <v>0.8376068376068376</v>
       </c>
     </row>
     <row r="10">
@@ -683,34 +683,34 @@
         </is>
       </c>
       <c r="B10" s="0" t="n">
-        <v>0.8436293436293436</v>
+        <v>0.694980694980695</v>
       </c>
       <c r="C10" s="0" t="n">
-        <v>0.9293154761904763</v>
+        <v>0.8630952380952381</v>
       </c>
       <c r="D10" s="0" t="n">
-        <v>0.8922784391534391</v>
+        <v>0.7959656084656084</v>
       </c>
       <c r="E10" s="0" t="n">
-        <v>0.8922784391534391</v>
+        <v>0.7959656084656084</v>
       </c>
       <c r="F10" s="0" t="n">
-        <v>0.8922784391534391</v>
+        <v>0.7959656084656084</v>
       </c>
       <c r="G10" s="0" t="n">
-        <v>0.8922784391534391</v>
+        <v>0.7959656084656084</v>
       </c>
       <c r="H10" s="0" t="n">
-        <v>0.8922784391534391</v>
+        <v>0.7959656084656084</v>
       </c>
       <c r="I10" s="0" t="n">
-        <v>0.8922784391534391</v>
+        <v>0.7959656084656084</v>
       </c>
       <c r="J10" s="0" t="n">
-        <v>0.8922784391534391</v>
+        <v>0.7959656084656084</v>
       </c>
       <c r="K10" s="0" t="n">
-        <v>0.8922784391534391</v>
+        <v>0.7959656084656084</v>
       </c>
     </row>
     <row r="11">
@@ -720,34 +720,34 @@
         </is>
       </c>
       <c r="B11" s="0" t="n">
-        <v>0.8502886002886003</v>
+        <v>0.7121212121212122</v>
       </c>
       <c r="C11" s="0" t="n">
-        <v>0.7256613756613757</v>
+        <v>0.5056437389770724</v>
       </c>
       <c r="D11" s="0" t="n">
-        <v>0.5194235588972431</v>
+        <v>0.25456498388829213</v>
       </c>
       <c r="E11" s="0" t="n">
-        <v>0.343003168003168</v>
+        <v>0.05770715770715772</v>
       </c>
       <c r="F11" s="0" t="n">
-        <v>0.34737588589809304</v>
+        <v>0.06119987274880262</v>
       </c>
       <c r="G11" s="0" t="n">
-        <v>0.402896450005086</v>
+        <v>0.12277489573797173</v>
       </c>
       <c r="H11" s="0" t="n">
-        <v>0.5066119471044231</v>
+        <v>0.21557227542179663</v>
       </c>
       <c r="I11" s="0" t="n">
-        <v>0.5370959194488607</v>
+        <v>0.23410174880763118</v>
       </c>
       <c r="J11" s="0" t="n">
-        <v>0.49955312455312456</v>
+        <v>0.1762655512655513</v>
       </c>
       <c r="K11" s="0" t="n">
-        <v>0.5724571078431373</v>
+        <v>0.27734375000000006</v>
       </c>
     </row>
     <row r="12">
@@ -757,34 +757,34 @@
         </is>
       </c>
       <c r="B12" s="0" t="n">
-        <v>0.8534883720930233</v>
+        <v>0.7255813953488373</v>
       </c>
       <c r="C12" s="0" t="n">
-        <v>0.7823529411764706</v>
+        <v>0.611764705882353</v>
       </c>
       <c r="D12" s="0" t="n">
-        <v>0.8534883720930233</v>
+        <v>0.7255813953488373</v>
       </c>
       <c r="E12" s="0" t="n">
-        <v>0.8534883720930233</v>
+        <v>0.7255813953488373</v>
       </c>
       <c r="F12" s="0" t="n">
-        <v>0.8534883720930233</v>
+        <v>0.7255813953488373</v>
       </c>
       <c r="G12" s="0" t="n">
-        <v>0.8534883720930233</v>
+        <v>0.7255813953488373</v>
       </c>
       <c r="H12" s="0" t="n">
-        <v>0.8534883720930233</v>
+        <v>0.7255813953488373</v>
       </c>
       <c r="I12" s="0" t="n">
-        <v>0.8534883720930233</v>
+        <v>0.7255813953488373</v>
       </c>
       <c r="J12" s="0" t="n">
-        <v>0.8534883720930233</v>
+        <v>0.7255813953488373</v>
       </c>
       <c r="K12" s="0" t="n">
-        <v>0.8534883720930233</v>
+        <v>0.7255813953488373</v>
       </c>
     </row>
     <row r="13">
@@ -794,34 +794,34 @@
         </is>
       </c>
       <c r="B13" s="0" t="n">
-        <v>0.828125</v>
+        <v>0.673828125</v>
       </c>
       <c r="C13" s="0" t="n">
-        <v>0.8040719696969697</v>
+        <v>0.6282196969696969</v>
       </c>
       <c r="D13" s="0" t="n">
-        <v>0.8040719696969697</v>
+        <v>0.6282196969696969</v>
       </c>
       <c r="E13" s="0" t="n">
-        <v>0.8040719696969697</v>
+        <v>0.6282196969696969</v>
       </c>
       <c r="F13" s="0" t="n">
-        <v>0.8040719696969697</v>
+        <v>0.6282196969696969</v>
       </c>
       <c r="G13" s="0" t="n">
-        <v>0.8040719696969697</v>
+        <v>0.6282196969696969</v>
       </c>
       <c r="H13" s="0" t="n">
-        <v>0.8040719696969697</v>
+        <v>0.6282196969696969</v>
       </c>
       <c r="I13" s="0" t="n">
-        <v>0.8040719696969697</v>
+        <v>0.6282196969696969</v>
       </c>
       <c r="J13" s="0" t="n">
-        <v>0.8040719696969697</v>
+        <v>0.6282196969696969</v>
       </c>
       <c r="K13" s="0" t="n">
-        <v>0.8040719696969697</v>
+        <v>0.6282196969696969</v>
       </c>
     </row>
     <row r="14">
@@ -831,34 +831,34 @@
         </is>
       </c>
       <c r="B14" s="0" t="n">
-        <v>0.9613095238095238</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="C14" s="0" t="n">
-        <v>0.9613095238095238</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="D14" s="0" t="n">
-        <v>0.9613095238095238</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="E14" s="0" t="n">
-        <v>0.9613095238095238</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="F14" s="0" t="n">
-        <v>0.9613095238095238</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="G14" s="0" t="n">
-        <v>0.9613095238095238</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="H14" s="0" t="n">
-        <v>0.9613095238095238</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="I14" s="0" t="n">
-        <v>0.9613095238095238</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="J14" s="0" t="n">
-        <v>0.9613095238095238</v>
+        <v>0.9226190476190477</v>
       </c>
       <c r="K14" s="0" t="n">
-        <v>0.9613095238095238</v>
+        <v>0.9226190476190477</v>
       </c>
     </row>
     <row r="15">

</xml_diff>